<commit_message>
All appendices alt text updated
</commit_message>
<xml_diff>
--- a/data/demo.xlsx
+++ b/data/demo.xlsx
@@ -414,7 +414,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="2">
-        <v>45916</v>
+        <v>45921</v>
       </c>
     </row>
     <row r="3">
@@ -438,7 +438,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="2">
-        <v>45915</v>
+        <v>45920</v>
       </c>
     </row>
     <row r="4">
@@ -462,7 +462,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="2">
-        <v>45914</v>
+        <v>45919</v>
       </c>
     </row>
     <row r="5">
@@ -486,7 +486,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="2">
-        <v>45913</v>
+        <v>45918</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +507,7 @@
         <v>5.5</v>
       </c>
       <c r="F6" s="2">
-        <v>45912</v>
+        <v>45917</v>
       </c>
     </row>
     <row r="7">
@@ -531,7 +531,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="2">
-        <v>45911</v>
+        <v>45916</v>
       </c>
     </row>
   </sheetData>

</xml_diff>